<commit_message>
Add independent enemy shields and hit-delayed recovery
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/battle_design.xlsx
+++ b/space-battleship/config_excel/battle_design.xlsx
@@ -1197,7 +1197,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>physical</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；physical仅为待验证目标</t>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>physical</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；energy仅为待验证目标</t>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>physical</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；physical仅为待验证目标</t>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>physical</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；energy仅为待验证目标</t>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add physical-attack pairs for the twenty enemy templates
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/battle_design.xlsx
+++ b/space-battleship/config_excel/battle_design.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,26 @@
           <t>description</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pair_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>attack_variant</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>attack_type</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>paired_group_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +529,26 @@
           <t>构成及测试条件说明</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>原版与变体共有的稳定模板标识</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>仅指敌方输出：energy_attack / physical_attack</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>敌方实际伤害类型：1能量/2物理；与counter所指防御克制独立</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>同模板另一攻击版本的monGroup ID</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -556,6 +596,26 @@
           <t>string</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -595,6 +655,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；laser仅为待验证目标</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>normal_laser</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>2001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -634,6 +710,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；missile仅为待验证目标</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>normal_missile</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2002</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -673,6 +765,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；cannon仅为待验证目标</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>normal_cannon</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2003</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -712,6 +820,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；longLaser仅为待验证目标</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>normal_longLaser</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>2004</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -751,6 +875,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral1仅为待验证目标</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>normal_neutral1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2005</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -790,6 +930,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral2仅为待验证目标</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>normal_neutral2</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2006</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -829,6 +985,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral3仅为待验证目标</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>normal_neutral3</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2007</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -868,6 +1040,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral4仅为待验证目标</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>normal_neutral4</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2008</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -907,6 +1095,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；laser仅为待验证目标</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>elite_laser</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>2009</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -946,6 +1150,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；missile仅为待验证目标</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>elite_missile</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2010</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -985,6 +1205,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；cannon仅为待验证目标</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>elite_cannon</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>2011</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1024,6 +1260,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；longLaser仅为待验证目标</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>elite_longLaser</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2012</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1063,6 +1315,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral1仅为待验证目标</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>elite_neutral1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="n">
+        <v>2013</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1102,6 +1370,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral2仅为待验证目标</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>elite_neutral2</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1141,6 +1425,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral3仅为待验证目标</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>elite_neutral3</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="n">
+        <v>2015</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1180,6 +1480,22 @@
           <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral4仅为待验证目标</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>elite_neutral4</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1219,6 +1535,22 @@
           <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>boss_physical</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1258,6 +1590,22 @@
           <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>boss_energy</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1297,6 +1645,22 @@
           <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>ultimate_physical</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1335,6 +1699,1122 @@
         <is>
           <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测</t>
         </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>ultimate_energy</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>energy_attack</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>normal_laser_physical_attack</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2001</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>laser</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；laser仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>normal_laser</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" t="n">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>normal_missile_physical_attack</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2002</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>missile</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>10</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>10</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；missile仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>normal_missile</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>2</v>
+      </c>
+      <c r="M25" t="n">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>normal_cannon_physical_attack</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2003</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>cannon</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>10</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>10</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；cannon仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>normal_cannon</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" t="n">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>normal_longLaser_physical_attack</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2004</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>longLaser</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；longLaser仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>normal_longLaser</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" t="n">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>normal_neutral1_physical_attack</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2005</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>10</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral1仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>normal_neutral1</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>normal_neutral2_physical_attack</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2006</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>10</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral2仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>normal_neutral2</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" t="n">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>normal_neutral3_physical_attack</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2007</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>10</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral3仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>normal_neutral3</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>2</v>
+      </c>
+      <c r="M30" t="n">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>normal_neutral4_physical_attack</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2008</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>normal</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>10</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>10</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral4仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>normal_neutral4</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="n">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>elite_laser_physical_attack</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2009</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>laser</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>20</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；laser仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>elite_laser</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="n">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>elite_missile_physical_attack</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2010</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>missile</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>10</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>20</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；missile仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>elite_missile</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>elite_cannon_physical_attack</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>cannon</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>10</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>20</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；cannon仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>elite_cannon</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>2</v>
+      </c>
+      <c r="M34" t="n">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>elite_longLaser_physical_attack</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2012</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>longLaser</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>10</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>20</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；longLaser仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>elite_longLaser</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>2</v>
+      </c>
+      <c r="M35" t="n">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>elite_neutral1_physical_attack</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2013</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>10</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" t="n">
+        <v>20</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral1仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>elite_neutral1</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>2</v>
+      </c>
+      <c r="M36" t="n">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>elite_neutral2_physical_attack</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2014</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>10</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="n">
+        <v>20</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral2仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>elite_neutral2</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>2</v>
+      </c>
+      <c r="M37" t="n">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>elite_neutral3_physical_attack</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2015</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>10</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>20</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral3仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>elite_neutral3</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L38" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" t="n">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>elite_neutral4_physical_attack</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>10</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>20</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>固定Destroyer四武器槽；护盾+护甲各一；Lv10+N；无额外加成；neutral4仅为待验证目标；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>elite_neutral4</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L39" t="n">
+        <v>2</v>
+      </c>
+      <c r="M39" t="n">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>boss_physical_physical_attack</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>10</v>
+      </c>
+      <c r="F40" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" t="n">
+        <v>30</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>boss_physical</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>2</v>
+      </c>
+      <c r="M40" t="n">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>boss_energy_physical_attack</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>physical</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>10</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" t="n">
+        <v>30</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>boss_energy</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L41" t="n">
+        <v>2</v>
+      </c>
+      <c r="M41" t="n">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ultimate_physical_physical_attack</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ultimate</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>10</v>
+      </c>
+      <c r="F42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G42" t="n">
+        <v>60</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>ultimate_physical</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>2</v>
+      </c>
+      <c r="M42" t="n">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ultimate_energy_physical_attack</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ultimate</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>physical</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>10</v>
+      </c>
+      <c r="F43" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" t="n">
+        <v>60</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>paired_template_pending</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>组名指敌方防御；counter仍指优势攻击类型；Destroyer Lv10+N，无额外加成；待实测；仅换敌方物理攻击，未完成新20组全量平衡验收。</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>ultimate_energy</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>physical_attack</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
+        <v>2</v>
+      </c>
+      <c r="M43" t="n">
+        <v>1020</v>
       </c>
     </row>
   </sheetData>

</xml_diff>